<commit_message>
feat: 딜러 등록 자동화에 Template Download·Region 자동 매핑 추가
임나연(해외영업1팀) 수정요청 3건 반영:
- Template Download 버튼(정식 DealerNET 템플릿)
- Member of Dealer 는 자동화 대상에서 제외 — "member of dealer" 헤더가
  기존 dealer 별칭에 잘못 매칭되던 문제를 PASSTHROUGH_ALIASES 로 차단
- 국가 원문 → HD Region(APAC/LA/MEA 등) 자동 판정 후 Account/Authorization
  Items to Select 26개를 제안(자동 제출 아님). permissions.json 의 국가
  코드 체계와는 분리해 절대 섞이지 않게 함
</commit_message>
<xml_diff>
--- a/sample/신규딜러_등록요청_20260826.xlsx
+++ b/sample/신규딜러_등록요청_20260826.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -745,6 +745,38 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Carlos Ruiz</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Guatemala</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Spanish</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>c.ruiz@centroam-eq.gt</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>CentroAm Equip.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>+502 2222 3333</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>